<commit_message>
Day 13 Update Drills
</commit_message>
<xml_diff>
--- a/outputs/day_13_trend_summary.xlsx
+++ b/outputs/day_13_trend_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t xml:space="preserve">accident_month</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">severity_adj_ma_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">severity_ma_12</t>
   </si>
   <si>
     <t xml:space="preserve">severity_linear_pred</t>
@@ -547,6 +550,9 @@
       <c r="S1" t="s">
         <v>18</v>
       </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -577,10 +583,10 @@
         <v>2022</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L2" t="n">
         <v>2738.87117873816</v>
@@ -594,10 +600,11 @@
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
-      <c r="R2" t="n">
+      <c r="R2"/>
+      <c r="S2" t="n">
         <v>2669.21080758057</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>2668.27391748223</v>
       </c>
     </row>
@@ -630,10 +637,10 @@
         <v>2022</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" t="n">
         <v>2568.33090129815</v>
@@ -647,10 +654,11 @@
       <c r="O3"/>
       <c r="P3"/>
       <c r="Q3"/>
-      <c r="R3" t="n">
+      <c r="R3"/>
+      <c r="S3" t="n">
         <v>2714.69200205075</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>2705.08366976576</v>
       </c>
     </row>
@@ -683,10 +691,10 @@
         <v>2022</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" t="n">
         <v>2527.91306769103</v>
@@ -704,10 +712,11 @@
       <c r="Q4" t="n">
         <v>2601.59338168617</v>
       </c>
-      <c r="R4" t="n">
+      <c r="R4"/>
+      <c r="S4" t="n">
         <v>2760.17319652094</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>2742.40122518534</v>
       </c>
     </row>
@@ -740,10 +749,10 @@
         <v>2022</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L5" t="n">
         <v>2546.83514964567</v>
@@ -761,10 +770,11 @@
       <c r="Q5" t="n">
         <v>2527.47499003183</v>
       </c>
-      <c r="R5" t="n">
+      <c r="R5"/>
+      <c r="S5" t="n">
         <v>2805.65439099112</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>2780.23358905912</v>
       </c>
     </row>
@@ -797,10 +807,10 @@
         <v>2022</v>
       </c>
       <c r="J6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L6" t="n">
         <v>2481.85255737782</v>
@@ -818,10 +828,11 @@
       <c r="Q6" t="n">
         <v>2488.95444034001</v>
       </c>
-      <c r="R6" t="n">
+      <c r="R6"/>
+      <c r="S6" t="n">
         <v>2851.1355854613</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>2818.58786334598</v>
       </c>
     </row>
@@ -854,10 +865,10 @@
         <v>2022</v>
       </c>
       <c r="J7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L7" t="n">
         <v>2697.22895269314</v>
@@ -877,10 +888,11 @@
       <c r="Q7" t="n">
         <v>2534.32619225083</v>
       </c>
-      <c r="R7" t="n">
+      <c r="R7"/>
+      <c r="S7" t="n">
         <v>2896.61677993149</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>2857.47124797877</v>
       </c>
     </row>
@@ -913,10 +925,10 @@
         <v>2022</v>
       </c>
       <c r="J8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L8" t="n">
         <v>2372.11127695111</v>
@@ -936,10 +948,11 @@
       <c r="Q8" t="n">
         <v>2467.477260977</v>
       </c>
-      <c r="R8" t="n">
+      <c r="R8"/>
+      <c r="S8" t="n">
         <v>2942.09797440167</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>2896.89104221588</v>
       </c>
     </row>
@@ -972,10 +985,10 @@
         <v>2022</v>
       </c>
       <c r="J9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L9" t="n">
         <v>3619.13458786848</v>
@@ -995,10 +1008,11 @@
       <c r="Q9" t="n">
         <v>2826.43195094649</v>
       </c>
-      <c r="R9" t="n">
+      <c r="R9"/>
+      <c r="S9" t="n">
         <v>2987.57916887185</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>2936.85464601145</v>
       </c>
     </row>
@@ -1031,10 +1045,10 @@
         <v>2022</v>
       </c>
       <c r="J10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L10" t="n">
         <v>3327.78669940675</v>
@@ -1054,10 +1068,11 @@
       <c r="Q10" t="n">
         <v>3019.51972975809</v>
       </c>
-      <c r="R10" t="n">
+      <c r="R10"/>
+      <c r="S10" t="n">
         <v>3033.06036334203</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>2977.36956140455</v>
       </c>
     </row>
@@ -1090,10 +1105,10 @@
         <v>2022</v>
       </c>
       <c r="J11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L11" t="n">
         <v>2556.91199587883</v>
@@ -1113,10 +1128,11 @@
       <c r="Q11" t="n">
         <v>3069.75581322249</v>
       </c>
-      <c r="R11" t="n">
+      <c r="R11"/>
+      <c r="S11" t="n">
         <v>3078.54155781222</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>3018.44339392742</v>
       </c>
     </row>
@@ -1149,10 +1165,10 @@
         <v>2022</v>
       </c>
       <c r="J12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L12" t="n">
         <v>4138.28594608572</v>
@@ -1172,10 +1188,11 @@
       <c r="Q12" t="n">
         <v>3222.06839781545</v>
       </c>
-      <c r="R12" t="n">
+      <c r="R12"/>
+      <c r="S12" t="n">
         <v>3124.0227522824</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>3060.08385403323</v>
       </c>
     </row>
@@ -1208,10 +1225,10 @@
         <v>2022</v>
       </c>
       <c r="J13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L13" t="n">
         <v>2876.67062623187</v>
@@ -1232,9 +1249,12 @@
         <v>3065.36636630643</v>
       </c>
       <c r="R13" t="n">
+        <v>2870.99441165556</v>
+      </c>
+      <c r="S13" t="n">
         <v>3169.50394675258</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>3102.2987585435</v>
       </c>
     </row>
@@ -1267,10 +1287,10 @@
         <v>2023</v>
       </c>
       <c r="J14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L14" t="n">
         <v>3357.98779141771</v>
@@ -1291,9 +1311,12 @@
         <v>3310.11323854872</v>
       </c>
       <c r="R14" t="n">
+        <v>2922.58746271219</v>
+      </c>
+      <c r="S14" t="n">
         <v>3214.98514122277</v>
       </c>
-      <c r="S14" t="n">
+      <c r="T14" t="n">
         <v>3145.09603211548</v>
       </c>
     </row>
@@ -1326,10 +1349,10 @@
         <v>2023</v>
       </c>
       <c r="J15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L15" t="n">
         <v>3100.82082673486</v>
@@ -1350,9 +1373,12 @@
         <v>2966.00170068347</v>
       </c>
       <c r="R15" t="n">
+        <v>2966.96162316525</v>
+      </c>
+      <c r="S15" t="n">
         <v>3260.46633569295</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>3188.48370872977</v>
       </c>
     </row>
@@ -1385,10 +1411,10 @@
         <v>2023</v>
       </c>
       <c r="J16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L16" t="n">
         <v>3263.66147989816</v>
@@ -1409,9 +1435,12 @@
         <v>3077.06217474991</v>
       </c>
       <c r="R16" t="n">
+        <v>3028.27399084918</v>
+      </c>
+      <c r="S16" t="n">
         <v>3305.94753016313</v>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>3232.46993319849</v>
       </c>
     </row>
@@ -1444,10 +1473,10 @@
         <v>2023</v>
       </c>
       <c r="J17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L17" t="n">
         <v>3210.00863562795</v>
@@ -1468,9 +1497,12 @@
         <v>3017.90085284832</v>
       </c>
       <c r="R17" t="n">
+        <v>3083.53844801437</v>
+      </c>
+      <c r="S17" t="n">
         <v>3351.42872463332</v>
       </c>
-      <c r="S17" t="n">
+      <c r="T17" t="n">
         <v>3277.06296269421</v>
       </c>
     </row>
@@ -1503,10 +1535,10 @@
         <v>2023</v>
       </c>
       <c r="J18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L18" t="n">
         <v>3249.99533994804</v>
@@ -1527,9 +1559,12 @@
         <v>3052.86652149924</v>
       </c>
       <c r="R18" t="n">
+        <v>3147.55034656189</v>
+      </c>
+      <c r="S18" t="n">
         <v>3396.9099191035</v>
       </c>
-      <c r="S18" t="n">
+      <c r="T18" t="n">
         <v>3322.27116830007</v>
       </c>
     </row>
@@ -1562,10 +1597,10 @@
         <v>2023</v>
       </c>
       <c r="J19" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L19" t="n">
         <v>3789.01079940506</v>
@@ -1586,9 +1621,12 @@
         <v>3204.24613052382</v>
       </c>
       <c r="R19" t="n">
+        <v>3238.53216712121</v>
+      </c>
+      <c r="S19" t="n">
         <v>3442.39111357368</v>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>3368.10303658112</v>
       </c>
     </row>
@@ -1621,10 +1659,10 @@
         <v>2023</v>
       </c>
       <c r="J20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L20" t="n">
         <v>3275.98015501926</v>
@@ -1645,9 +1683,12 @@
         <v>3212.71428752473</v>
       </c>
       <c r="R20" t="n">
+        <v>3313.85457362689</v>
+      </c>
+      <c r="S20" t="n">
         <v>3487.87230804387</v>
       </c>
-      <c r="S20" t="n">
+      <c r="T20" t="n">
         <v>3414.56717117751</v>
       </c>
     </row>
@@ -1680,10 +1721,10 @@
         <v>2023</v>
       </c>
       <c r="J21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L21" t="n">
         <v>6092.68530290303</v>
@@ -1704,9 +1745,12 @@
         <v>4078.96578831705</v>
       </c>
       <c r="R21" t="n">
+        <v>3519.98379987977</v>
+      </c>
+      <c r="S21" t="n">
         <v>3533.35350251405</v>
       </c>
-      <c r="S21" t="n">
+      <c r="T21" t="n">
         <v>3461.67229441954</v>
       </c>
     </row>
@@ -1739,10 +1783,10 @@
         <v>2023</v>
       </c>
       <c r="J22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L22" t="n">
         <v>2902.93651851942</v>
@@ -1763,9 +1807,12 @@
         <v>3792.22332187982</v>
       </c>
       <c r="R22" t="n">
+        <v>3484.57961813916</v>
+      </c>
+      <c r="S22" t="n">
         <v>3578.83469698423</v>
       </c>
-      <c r="S22" t="n">
+      <c r="T22" t="n">
         <v>3509.42724896504</v>
       </c>
     </row>
@@ -1798,10 +1845,10 @@
         <v>2023</v>
       </c>
       <c r="J23" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L23" t="n">
         <v>3694.61481237262</v>
@@ -1822,9 +1869,12 @@
         <v>3908.44831268318</v>
       </c>
       <c r="R23" t="n">
+        <v>3579.38818618031</v>
+      </c>
+      <c r="S23" t="n">
         <v>3624.31589145441</v>
       </c>
-      <c r="S23" t="n">
+      <c r="T23" t="n">
         <v>3557.84099945935</v>
       </c>
     </row>
@@ -1857,10 +1907,10 @@
         <v>2023</v>
       </c>
       <c r="J24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L24" t="n">
         <v>3578.34898534561</v>
@@ -1881,9 +1931,12 @@
         <v>3118.39220637028</v>
       </c>
       <c r="R24" t="n">
+        <v>3532.7267727853</v>
+      </c>
+      <c r="S24" t="n">
         <v>3669.7970859246</v>
       </c>
-      <c r="S24" t="n">
+      <c r="T24" t="n">
         <v>3606.92263421813</v>
       </c>
     </row>
@@ -1916,10 +1969,10 @@
         <v>2023</v>
       </c>
       <c r="J25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L25" t="n">
         <v>3655.57954906039</v>
@@ -1940,9 +1993,12 @@
         <v>3336.62855832306</v>
       </c>
       <c r="R25" t="n">
+        <v>3597.63584968768</v>
+      </c>
+      <c r="S25" t="n">
         <v>3715.27828039478</v>
       </c>
-      <c r="S25" t="n">
+      <c r="T25" t="n">
         <v>3656.6813669335</v>
       </c>
     </row>
@@ -1975,10 +2031,10 @@
         <v>2024</v>
       </c>
       <c r="J26" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L26" t="n">
         <v>3757.87381896596</v>
@@ -1999,9 +2055,12 @@
         <v>3342.30634967875</v>
       </c>
       <c r="R26" t="n">
+        <v>3630.9596853167</v>
+      </c>
+      <c r="S26" t="n">
         <v>3760.75947486496</v>
       </c>
-      <c r="S26" t="n">
+      <c r="T26" t="n">
         <v>3707.12653840361</v>
       </c>
     </row>
@@ -2034,10 +2093,10 @@
         <v>2024</v>
       </c>
       <c r="J27" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L27" t="n">
         <v>3494.18679141174</v>
@@ -2058,9 +2117,12 @@
         <v>3303.9111539157</v>
       </c>
       <c r="R27" t="n">
+        <v>3663.7401823731</v>
+      </c>
+      <c r="S27" t="n">
         <v>3806.24066933515</v>
       </c>
-      <c r="S27" t="n">
+      <c r="T27" t="n">
         <v>3758.26761828609</v>
       </c>
     </row>
@@ -2093,10 +2155,10 @@
         <v>2024</v>
       </c>
       <c r="J28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K28" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L28" t="n">
         <v>3598.3774157157</v>
@@ -2117,9 +2179,12 @@
         <v>3273.49005523225</v>
       </c>
       <c r="R28" t="n">
+        <v>3691.63317702457</v>
+      </c>
+      <c r="S28" t="n">
         <v>3851.72186380533</v>
       </c>
-      <c r="S28" t="n">
+      <c r="T28" t="n">
         <v>3810.11420687578</v>
       </c>
     </row>
@@ -2152,10 +2217,10 @@
         <v>2024</v>
       </c>
       <c r="J29" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L29" t="n">
         <v>3403.49861591252</v>
@@ -2176,9 +2241,12 @@
         <v>3153.88524379454</v>
       </c>
       <c r="R29" t="n">
+        <v>3707.75734204828</v>
+      </c>
+      <c r="S29" t="n">
         <v>3897.20305827551</v>
       </c>
-      <c r="S29" t="n">
+      <c r="T29" t="n">
         <v>3862.67603690684</v>
       </c>
     </row>
@@ -2211,10 +2279,10 @@
         <v>2024</v>
       </c>
       <c r="J30" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K30" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L30" t="n">
         <v>4630.32864549029</v>
@@ -2235,9 +2303,12 @@
         <v>3479.9992439165</v>
       </c>
       <c r="R30" t="n">
+        <v>3822.78511751013</v>
+      </c>
+      <c r="S30" t="n">
         <v>3942.6842527457</v>
       </c>
-      <c r="S30" t="n">
+      <c r="T30" t="n">
         <v>3915.96297537986</v>
       </c>
     </row>
@@ -2270,10 +2341,10 @@
         <v>2024</v>
       </c>
       <c r="J31" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L31" t="n">
         <v>3956.23502449149</v>
@@ -2294,9 +2365,12 @@
         <v>3573.37355768055</v>
       </c>
       <c r="R31" t="n">
+        <v>3836.72046960067</v>
+      </c>
+      <c r="S31" t="n">
         <v>3988.16544721588</v>
       </c>
-      <c r="S31" t="n">
+      <c r="T31" t="n">
         <v>3969.98502541407</v>
       </c>
     </row>
@@ -2329,10 +2403,10 @@
         <v>2024</v>
       </c>
       <c r="J32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L32" t="n">
         <v>4051.8734225203</v>
@@ -2353,9 +2427,12 @@
         <v>3752.97927308224</v>
       </c>
       <c r="R32" t="n">
+        <v>3901.37824189242</v>
+      </c>
+      <c r="S32" t="n">
         <v>4033.64664168606</v>
       </c>
-      <c r="S32" t="n">
+      <c r="T32" t="n">
         <v>4024.75232812513</v>
       </c>
     </row>
@@ -2388,10 +2465,10 @@
         <v>2024</v>
       </c>
       <c r="J33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L33" t="n">
         <v>3958.55147935568</v>
@@ -2412,9 +2489,12 @@
         <v>3538.6879193529</v>
       </c>
       <c r="R33" t="n">
+        <v>3723.53375659681</v>
+      </c>
+      <c r="S33" t="n">
         <v>4079.12783615624</v>
       </c>
-      <c r="S33" t="n">
+      <c r="T33" t="n">
         <v>4080.2751645289</v>
       </c>
     </row>
@@ -2447,10 +2527,10 @@
         <v>2024</v>
       </c>
       <c r="J34" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K34" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L34" t="n">
         <v>4307.79361375791</v>
@@ -2471,9 +2551,12 @@
         <v>3627.83795330207</v>
       </c>
       <c r="R34" t="n">
+        <v>3840.60518120002</v>
+      </c>
+      <c r="S34" t="n">
         <v>4124.60903062643</v>
       </c>
-      <c r="S34" t="n">
+      <c r="T34" t="n">
         <v>4136.56395747135</v>
       </c>
     </row>
@@ -2506,10 +2589,10 @@
         <v>2024</v>
       </c>
       <c r="J35" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K35" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L35" t="n">
         <v>4747.5296399695</v>
@@ -2530,9 +2613,12 @@
         <v>3816.83821737671</v>
       </c>
       <c r="R35" t="n">
+        <v>3928.34808349976</v>
+      </c>
+      <c r="S35" t="n">
         <v>4170.09022509661</v>
       </c>
-      <c r="S35" t="n">
+      <c r="T35" t="n">
         <v>4193.6292735852</v>
       </c>
     </row>
@@ -2565,10 +2651,10 @@
         <v>2024</v>
       </c>
       <c r="J36" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L36" t="n">
         <v>3903.13909188021</v>
@@ -2589,9 +2675,12 @@
         <v>3786.8318536301</v>
       </c>
       <c r="R36" t="n">
+        <v>3955.41392571097</v>
+      </c>
+      <c r="S36" t="n">
         <v>4215.57141956679</v>
       </c>
-      <c r="S36" t="n">
+      <c r="T36" t="n">
         <v>4251.48182527348</v>
       </c>
     </row>
@@ -2624,10 +2713,10 @@
         <v>2024</v>
       </c>
       <c r="J37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L37" t="n">
         <v>3311.79089352572</v>
@@ -2648,9 +2737,12 @@
         <v>3483.07925486568</v>
       </c>
       <c r="R37" t="n">
+        <v>3926.76487108308</v>
+      </c>
+      <c r="S37" t="n">
         <v>4261.05261403698</v>
       </c>
-      <c r="S37" t="n">
+      <c r="T37" t="n">
         <v>4310.13247272045</v>
       </c>
     </row>
@@ -2670,13 +2762,13 @@
         <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
         <v>11</v>
@@ -2687,7 +2779,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" t="n">
         <v>251</v>
@@ -2707,7 +2799,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" t="n">
         <v>268</v>
@@ -2727,7 +2819,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" t="n">
         <v>247</v>
@@ -2747,7 +2839,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" t="n">
         <v>275</v>
@@ -2767,7 +2859,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" t="n">
         <v>274</v>
@@ -2787,7 +2879,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B7" t="n">
         <v>284</v>
@@ -2807,7 +2899,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" t="n">
         <v>281</v>
@@ -2827,7 +2919,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" t="n">
         <v>279</v>
@@ -2847,7 +2939,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" t="n">
         <v>290</v>
@@ -2867,7 +2959,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" t="n">
         <v>312</v>
@@ -2887,7 +2979,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12" t="n">
         <v>325</v>
@@ -2907,7 +2999,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" t="n">
         <v>343</v>
@@ -2938,46 +3030,46 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" t="n">
         <v>45.4811944701831</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B3" t="n">
         <v>0.0137953423905801</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" t="n">
         <v>0.178700586738551</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>